<commit_message>
data: backfill Channel column in AR_Tracking sheet
</commit_message>
<xml_diff>
--- a/PTH_progress_tracking.xlsx
+++ b/PTH_progress_tracking.xlsx
@@ -56643,7 +56643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -56654,30 +56654,35 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Channel</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>ETA</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Remark</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -56691,30 +56696,35 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>Teams</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>Hello Everyone, I have listed all the open items still under active debug and implementation. Please check and update...</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Kandhan</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Please check and update if anything missed. This will be reviewed with Yonghyun on Wednesday. | From: Basavaraju, Kamalesh</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>4c7590c05a7c</t>
         </is>
@@ -56728,30 +56738,35 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>Teams</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>can you share the CFC data by tomorrow</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Ranganathan, Saravanann</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>can you share the CFC data by tomorrow | From: Rajakumar, Kandhan</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>82ad113ce473</t>
         </is>
@@ -56765,30 +56780,35 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>Teams</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>Hi Panigrahy, Bisweswar , Maji, Debabrata , Rajakumar, Kandhan , Mathew, Jayson , Mallya K, Harish , Parameshwari, Me...</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Kandhan</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>xlsx please update the tracker page as of today by 11AM Tomorrow. | From: Kodandaramaiah, Chandrashekar</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>9a623f95a832</t>
         </is>
@@ -56802,30 +56822,35 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>Teams</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>can you discuss with me while in office</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Balakrishnan, SankkaraX Naarayanan</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>can you discuss with me while in office | From: Rajakumar, Kandhan</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>a8a8420e94a1</t>
         </is>
@@ -56839,30 +56864,35 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>Teams</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>by EOD can you able to share</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Anand, RishiX</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>by EOD can you able to share | From: Rajakumar, Kandhan</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>f5c55ae119a8</t>
         </is>
@@ -56876,30 +56906,35 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>Teams</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>and can you plot dts plot as like earlier</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Anand, RishiX</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>and can you plot dts plot as like earlier | From: Rajakumar, Kandhan</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>94f4e2cd6dea</t>
         </is>
@@ -56913,30 +56948,35 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>Teams</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>can you give me the excel with full read read</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Anand, RishiX</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>can you give me the excel with full read read | From: Rajakumar, Kandhan</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>f898e5a47646</t>
         </is>
@@ -56950,30 +56990,35 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>Outlook</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>Collective and individual reports on takeaway, action plan based on ITC - Participation</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Kandhan</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Q3/Q4</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>We need to have a Plan for Q3/Q4 realization of the takeaways and implement them and showcase. | From: chandrashekhar.m.v@intel.com</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>41e496aa99a3</t>
         </is>
@@ -56987,30 +57032,35 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>Teams</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>Everyone MO's please fill you CW's tasks in sheet daily basis</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Kandhan</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Everyone MO's please fill you CW's tasks in sheet daily basis | From: Singh, Partap</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>ba27a4baf121</t>
         </is>
@@ -57024,30 +57074,35 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>Teams</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>can you setup meeting tomorrow</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Balakrishnan, SankkaraX Naarayanan</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>can you setup meeting tomorrow | From: Rajakumar, Kandhan</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>fe9e248d1bfa</t>
         </is>
@@ -57061,30 +57116,35 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>Teams</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
           <t>BA AI initiatives- Summary - ww30.3.pptx shared to management. Please review and let us know if any inputs.</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Kandhan</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>WW30.3</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>BA AI initiatives- Summary - ww30.3.pptx shared to management. Please review and let us know if any inputs. | From: Kodandaramaiah, Chandrashekar</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>644c96a29f54</t>
         </is>
@@ -57098,30 +57158,35 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>Teams</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
           <t>Anand, Harsh can you figure out the issue</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Anand, RishiX</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>Anand, Harsh can you figure out the issue | From: Rajakumar, Kandhan</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>2af3f93e4cfa</t>
         </is>
@@ -57135,30 +57200,35 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>Teams</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
           <t>Aneesh K A Babu Kumar, AnjuX please join</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Kandhan</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>Aneesh K A Babu Kumar, AnjuX please join | From: Singh, Partap</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>e8955967df12</t>
         </is>
@@ -57172,32 +57242,79 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
+          <t>Teams</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
           <t>Hi Panigrahy, Bisweswar , Maji, Debabrata , Rajakumar, Kandhan , Mathew, Jayson , Mallya K, Harish , Parameshwari, Me...</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>Kandhan</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>xlsx please update the tracker page as of today by 11AM today. | From: Kodandaramaiah, Chandrashekar</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>c4d7f79dfdfa</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Outlook</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Re: [Action Required] GNR-D XCC+ Program Audit w.r.t. GNR-D HCC and GND-SP XCC – Request for Module-Level Review</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>We went over what we intercepted/learned in the middle of GNR-SP execution, and everything seemed to | From: joseph.a.blanco.fallas@intel.com</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>d18838414214</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add sent-mail follow-up ARs to AR_Tracking (5 rows)
</commit_message>
<xml_diff>
--- a/PTH_progress_tracking.xlsx
+++ b/PTH_progress_tracking.xlsx
@@ -56643,7 +56643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -57318,6 +57318,216 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07-28</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Outlook</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Provide GNRD XCCP A0 Efficiency FER and FSL data for review</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Ranganathan, Saravanann</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>WW30</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Kandhan follow-up: please provide the data by this week | Thread: GNRD XCCP A0 Efficiency FER, FSL data review | From: kandhan.rajakumar@intel.com</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Outlook:2d0c5de8c883</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Outlook</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Provide updated IA FSL S2T multiplier for 10% guard band (GNR-D XCC+ power failure improvement)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Krishnan, Rohini</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Kandhan asked Rohini: calculate IA FSL S2T multiplier when reducing GB from 20% to 10% for GNR-D XCC+ | From: kandhan.rajakumar@intel.com</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Outlook:c24becca4c76</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Outlook</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Share noted differences from GNR-D XCC+ Program Audit (vs GNR-D HCC and GND-SP XCC)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Rivera Valverde, Pablo</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Kandhan asked Pablo to share noted differences from GNR-D XCC+ module-level audit review | From: kandhan.rajakumar@intel.com</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Outlook:c6b98c0d2912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Outlook</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Help with 10% IA FSL S2T multiplier (1.1) calculation for GNR-D XCC+ power failure improvement path</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Ranganathan, Saravanann</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Kandhan asked Saravanan to help calculate 10% IA FSL S2T multiplier (value: 1.1) per Maji request | From: kandhan.rajakumar@intel.com</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Outlook:ec6050b1d005</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-07-14</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Outlook</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>File JIRA ticket to Prime team for Bin2719 offset calculation error (GNR-D XCC+ CLASSHOT yield)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Kandhan</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Bin2719 failing due to Prime template offset calculation bug (not silicon). Kandhan to file JIRA with Prime team. DOEs ongoing. | From: kandhan.rajakumar@intel.com</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Outlook:f3e8d099349d</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: readable Source column (Outlook:Inbox/Sent/Search, Teams), sent-mail ARs, doc updates
</commit_message>
<xml_diff>
--- a/PTH_progress_tracking.xlsx
+++ b/PTH_progress_tracking.xlsx
@@ -56691,22 +56691,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Teams</t>
+          <t>Outlook:Inbox</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hello Everyone, I have listed all the open items still under active debug and implementation. Please check and update...</t>
+          <t>Re: [Action Required] GNR-D XCC+ Program Audit w.r.t. GNR-D HCC and GND-SP XCC – Request for Module-Level Review</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Kandhan</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -56721,12 +56721,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Please check and update if anything missed. This will be reviewed with Yonghyun on Wednesday. | From: Basavaraju, Kamalesh</t>
+          <t>We went over what we intercepted/learned in the middle of GNR-SP execution, and everything seemed to | From: joseph.a.blanco.fallas@intel.com</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>4c7590c05a7c</t>
+          <t>Outlook:Inbox:d18838414214</t>
         </is>
       </c>
     </row>
@@ -56743,12 +56743,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>can you share the CFC data by tomorrow</t>
+          <t>Hello Everyone, I have listed all the open items still under active debug and implementation. Please check and update...</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Ranganathan, Saravanann</t>
+          <t>Kandhan</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -56763,12 +56763,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>can you share the CFC data by tomorrow | From: Rajakumar, Kandhan</t>
+          <t>Please check and update if anything missed. This will be reviewed with Yonghyun on Wednesday. | From: Basavaraju, Kamalesh</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>82ad113ce473</t>
+          <t>Teams:4c7590c05a7c</t>
         </is>
       </c>
     </row>
@@ -56785,12 +56785,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Hi Panigrahy, Bisweswar , Maji, Debabrata , Rajakumar, Kandhan , Mathew, Jayson , Mallya K, Harish , Parameshwari, Me...</t>
+          <t>can you share the CFC data by tomorrow</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Kandhan</t>
+          <t>Ranganathan, Saravanann</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -56805,12 +56805,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>xlsx please update the tracker page as of today by 11AM Tomorrow. | From: Kodandaramaiah, Chandrashekar</t>
+          <t>can you share the CFC data by tomorrow | From: Rajakumar, Kandhan</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>9a623f95a832</t>
+          <t>Teams:82ad113ce473</t>
         </is>
       </c>
     </row>
@@ -56827,12 +56827,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>can you discuss with me while in office</t>
+          <t>Hi Panigrahy, Bisweswar , Maji, Debabrata , Rajakumar, Kandhan , Mathew, Jayson , Mallya K, Harish , Parameshwari, Me...</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Balakrishnan, SankkaraX Naarayanan</t>
+          <t>Kandhan</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -56847,19 +56847,19 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>can you discuss with me while in office | From: Rajakumar, Kandhan</t>
+          <t>xlsx please update the tracker page as of today by 11AM Tomorrow. | From: Kodandaramaiah, Chandrashekar</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>a8a8420e94a1</t>
+          <t>Teams:9a623f95a832</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -56869,12 +56869,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>by EOD can you able to share</t>
+          <t>can you discuss with me while in office</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Anand, RishiX</t>
+          <t>Balakrishnan, SankkaraX Naarayanan</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -56889,12 +56889,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>by EOD can you able to share | From: Rajakumar, Kandhan</t>
+          <t>can you discuss with me while in office | From: Rajakumar, Kandhan</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>f5c55ae119a8</t>
+          <t>Teams:a8a8420e94a1</t>
         </is>
       </c>
     </row>
@@ -56911,7 +56911,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>and can you plot dts plot as like earlier</t>
+          <t>by EOD can you able to share</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -56931,12 +56931,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>and can you plot dts plot as like earlier | From: Rajakumar, Kandhan</t>
+          <t>by EOD can you able to share | From: Rajakumar, Kandhan</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>94f4e2cd6dea</t>
+          <t>Teams:f5c55ae119a8</t>
         </is>
       </c>
     </row>
@@ -56953,7 +56953,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>can you give me the excel with full read read</t>
+          <t>and can you plot dts plot as like earlier</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -56973,12 +56973,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>can you give me the excel with full read read | From: Rajakumar, Kandhan</t>
+          <t>and can you plot dts plot as like earlier | From: Rajakumar, Kandhan</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>f898e5a47646</t>
+          <t>Teams:94f4e2cd6dea</t>
         </is>
       </c>
     </row>
@@ -56990,17 +56990,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Outlook</t>
+          <t>Teams</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Collective and individual reports on takeaway, action plan based on ITC - Participation</t>
+          <t>can you give me the excel with full read read</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Kandhan</t>
+          <t>Anand, RishiX</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -57010,17 +57010,17 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Q3/Q4</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>We need to have a Plan for Q3/Q4 realization of the takeaways and implement them and showcase. | From: chandrashekhar.m.v@intel.com</t>
+          <t>can you give me the excel with full read read | From: Rajakumar, Kandhan</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>41e496aa99a3</t>
+          <t>Teams:f898e5a47646</t>
         </is>
       </c>
     </row>
@@ -57032,12 +57032,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Teams</t>
+          <t>Outlook:Search</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Everyone MO's please fill you CW's tasks in sheet daily basis</t>
+          <t>Collective and individual reports on takeaway, action plan based on ITC - Participation</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -57052,24 +57052,24 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Q3/Q4</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Everyone MO's please fill you CW's tasks in sheet daily basis | From: Singh, Partap</t>
+          <t>We need to have a Plan for Q3/Q4 realization of the takeaways and implement them and showcase. | From: chandrashekhar.m.v@intel.com</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>ba27a4baf121</t>
+          <t>Outlook:Search:41e496aa99a3</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -57079,12 +57079,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>can you setup meeting tomorrow</t>
+          <t>Everyone MO's please fill you CW's tasks in sheet daily basis</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Balakrishnan, SankkaraX Naarayanan</t>
+          <t>Kandhan</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -57099,12 +57099,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>can you setup meeting tomorrow | From: Rajakumar, Kandhan</t>
+          <t>Everyone MO's please fill you CW's tasks in sheet daily basis | From: Singh, Partap</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>fe9e248d1bfa</t>
+          <t>Teams:ba27a4baf121</t>
         </is>
       </c>
     </row>
@@ -57121,12 +57121,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BA AI initiatives- Summary - ww30.3.pptx shared to management. Please review and let us know if any inputs.</t>
+          <t>can you setup meeting tomorrow</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Kandhan</t>
+          <t>Balakrishnan, SankkaraX Naarayanan</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -57136,17 +57136,17 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>WW30.3</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>BA AI initiatives- Summary - ww30.3.pptx shared to management. Please review and let us know if any inputs. | From: Kodandaramaiah, Chandrashekar</t>
+          <t>can you setup meeting tomorrow | From: Rajakumar, Kandhan</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>644c96a29f54</t>
+          <t>Teams:fe9e248d1bfa</t>
         </is>
       </c>
     </row>
@@ -57163,12 +57163,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Anand, Harsh can you figure out the issue</t>
+          <t>BA AI initiatives- Summary - ww30.3.pptx shared to management. Please review and let us know if any inputs.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Anand, RishiX</t>
+          <t>Kandhan</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -57178,17 +57178,17 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>WW30.3</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Anand, Harsh can you figure out the issue | From: Rajakumar, Kandhan</t>
+          <t>BA AI initiatives- Summary - ww30.3.pptx shared to management. Please review and let us know if any inputs. | From: Kodandaramaiah, Chandrashekar</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>2af3f93e4cfa</t>
+          <t>Teams:644c96a29f54</t>
         </is>
       </c>
     </row>
@@ -57205,12 +57205,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Aneesh K A Babu Kumar, AnjuX please join</t>
+          <t>Anand, Harsh can you figure out the issue</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Kandhan</t>
+          <t>Anand, RishiX</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -57225,12 +57225,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Aneesh K A Babu Kumar, AnjuX please join | From: Singh, Partap</t>
+          <t>Anand, Harsh can you figure out the issue | From: Rajakumar, Kandhan</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>e8955967df12</t>
+          <t>Teams:2af3f93e4cfa</t>
         </is>
       </c>
     </row>
@@ -57247,7 +57247,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Hi Panigrahy, Bisweswar , Maji, Debabrata , Rajakumar, Kandhan , Mathew, Jayson , Mallya K, Harish , Parameshwari, Me...</t>
+          <t>Aneesh K A Babu Kumar, AnjuX please join</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -57267,54 +57267,54 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>xlsx please update the tracker page as of today by 11AM today. | From: Kodandaramaiah, Chandrashekar</t>
+          <t>Aneesh K A Babu Kumar, AnjuX please join | From: Singh, Partap</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>c4d7f79dfdfa</t>
+          <t>Teams:e8955967df12</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Outlook</t>
+          <t>Teams</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Re: [Action Required] GNR-D XCC+ Program Audit w.r.t. GNR-D HCC and GND-SP XCC – Request for Module-Level Review</t>
+          <t>Hi Panigrahy, Bisweswar , Maji, Debabrata , Rajakumar, Kandhan , Mathew, Jayson , Mallya K, Harish , Parameshwari, Me...</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
+          <t>Kandhan</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
           <t>TBD</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>Open</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>We went over what we intercepted/learned in the middle of GNR-SP execution, and everything seemed to | From: joseph.a.blanco.fallas@intel.com</t>
+          <t>xlsx please update the tracker page as of today by 11AM today. | From: Kodandaramaiah, Chandrashekar</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>d18838414214</t>
+          <t>Teams:c4d7f79dfdfa</t>
         </is>
       </c>
     </row>
@@ -57326,7 +57326,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Outlook</t>
+          <t>Outlook:Sent</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -57356,7 +57356,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Outlook:2d0c5de8c883</t>
+          <t>Outlook:Sent:2d0c5de8c883</t>
         </is>
       </c>
     </row>
@@ -57368,7 +57368,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Outlook</t>
+          <t>Outlook:Sent</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -57398,7 +57398,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Outlook:c24becca4c76</t>
+          <t>Outlook:Sent:c24becca4c76</t>
         </is>
       </c>
     </row>
@@ -57410,7 +57410,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Outlook</t>
+          <t>Outlook:Sent</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -57440,7 +57440,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Outlook:c6b98c0d2912</t>
+          <t>Outlook:Sent:c6b98c0d2912</t>
         </is>
       </c>
     </row>
@@ -57452,7 +57452,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Outlook</t>
+          <t>Outlook:Sent</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -57482,7 +57482,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Outlook:ec6050b1d005</t>
+          <t>Outlook:Sent:ec6050b1d005</t>
         </is>
       </c>
     </row>
@@ -57494,7 +57494,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Outlook</t>
+          <t>Outlook:Sent</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -57524,7 +57524,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Outlook:f3e8d099349d</t>
+          <t>Outlook:Sent:f3e8d099349d</t>
         </is>
       </c>
     </row>

</xml_diff>